<commit_message>
Restructure adobe-partner landing into 3 styled sections
cms-dam (and the shared adobe-partner-landing template) imported as one
flat section. Split it into the three source bands with their shells:
- hero (bg-pn), "why" (bg-pn-second), tools (bg-pn) via section metadata
- add a reusable title-page block (blue accent line; variants line-top
  center 41px / line-bottom left small 20px) + its import parser for the
  centered section titles
- cards-benefits: transparent two-column "why" layout, column subtitles
  get the blue underline
- cards-solution: translucent dark product cards in a 3-column grid with
  cyan hover

cms-dam completeness 26%→97.7%. Content regenerated via the import
pipeline (content/ is git-ignored).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-adobe-partner-landing.report.xlsx
+++ b/tools/importer/reports/import-adobe-partner-landing.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="71">
   <si>
     <t>_reportFile</t>
   </si>
@@ -37,25 +37,58 @@
     <t>url</t>
   </si>
   <si>
+    <t>blog.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","blog-list"]</t>
+  </si>
+  <si>
+    <t>blog</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>blog-listing</t>
+  </si>
+  <si>
+    <t>2026-08-25T23:56:14.319Z</t>
+  </si>
+  <si>
+    <t>Ecosistema Adobe dentro de Puntos.net</t>
+  </si>
+  <si>
+    <t>http://adobe.puntos.net.s3-website-us-east-1.amazonaws.com/blog</t>
+  </si>
+  <si>
+    <t>contacto.report.json</t>
+  </si>
+  <si>
+    <t>["contact-form","contact-form","contact-form"]</t>
+  </si>
+  <si>
+    <t>contacto</t>
+  </si>
+  <si>
+    <t>2026-09-10T16:20:46.462Z</t>
+  </si>
+  <si>
+    <t>http://adobe.puntos.net.s3-website-us-east-1.amazonaws.com/contacto</t>
+  </si>
+  <si>
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["hero-partner","cards-stats","cards-product"]</t>
+    <t>["home-ecosystem"]</t>
   </si>
   <si>
     <t>index</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
     <t>home</t>
   </si>
   <si>
-    <t>2026-08-25T23:55:20.207Z</t>
-  </si>
-  <si>
-    <t>Ecosistema Adobe dentro de Puntos.net</t>
+    <t>2026-09-10T04:52:43.408Z</t>
   </si>
   <si>
     <t>http://adobe.puntos.net.s3-website-us-east-1.amazonaws.com/</t>
@@ -64,7 +97,7 @@
     <t>adobe-partner/arquitectura-headless.report.json</t>
   </si>
   <si>
-    <t>["hero-partner"]</t>
+    <t>["hero-partner","title-page","title-page","title-page"]</t>
   </si>
   <si>
     <t>adobe-partner/arquitectura-headless</t>
@@ -73,7 +106,7 @@
     <t>adobe-partner-landing</t>
   </si>
   <si>
-    <t>2026-08-25T23:55:53.529Z</t>
+    <t>2026-09-10T23:44:40.957Z</t>
   </si>
   <si>
     <t>http://adobe.puntos.net.s3-website-us-east-1.amazonaws.com/adobe-partner/arquitectura-headless</t>
@@ -88,7 +121,7 @@
     <t>adobe-partner/automatizacion-omnicanal</t>
   </si>
   <si>
-    <t>2026-08-25T23:56:06.564Z</t>
+    <t>2026-09-10T23:44:52.607Z</t>
   </si>
   <si>
     <t>http://adobe.puntos.net.s3-website-us-east-1.amazonaws.com/adobe-partner/automatizacion-omnicanal</t>
@@ -97,13 +130,13 @@
     <t>adobe-partner/cms-dam.report.json</t>
   </si>
   <si>
-    <t>["hero-partner","cards-benefits","cards-benefits","cards-benefits","cards-benefits","cards-benefits","cards-benefits","cards-solution","cards-solution","cards-solution","cards-solution","cards-solution","cards-solution","cards-solution"]</t>
+    <t>["hero-partner","title-page","title-page","cards-benefits","cards-benefits","cards-benefits","cards-benefits","cards-benefits","cards-benefits","cards-solution","cards-solution","cards-solution","cards-solution","cards-solution","cards-solution","cards-solution"]</t>
   </si>
   <si>
     <t>adobe-partner/cms-dam</t>
   </si>
   <si>
-    <t>2026-08-25T23:55:35.411Z</t>
+    <t>2026-09-10T23:44:20.288Z</t>
   </si>
   <si>
     <t>http://adobe.puntos.net.s3-website-us-east-1.amazonaws.com/adobe-partner/cms-dam</t>
@@ -115,7 +148,7 @@
     <t>adobe-partner/datos-accionables</t>
   </si>
   <si>
-    <t>2026-08-25T23:55:46.460Z</t>
+    <t>2026-09-10T23:44:34.102Z</t>
   </si>
   <si>
     <t>http://adobe.puntos.net.s3-website-us-east-1.amazonaws.com/adobe-partner/datos-accionables</t>
@@ -127,7 +160,7 @@
     <t>adobe-partner/mail-marketing</t>
   </si>
   <si>
-    <t>2026-08-25T23:56:00.798Z</t>
+    <t>2026-09-10T23:44:45.975Z</t>
   </si>
   <si>
     <t>http://adobe.puntos.net.s3-website-us-east-1.amazonaws.com/adobe-partner/mail-marketing</t>
@@ -139,10 +172,58 @@
     <t>adobe-partner/personalizacion</t>
   </si>
   <si>
-    <t>2026-08-25T23:55:40.714Z</t>
+    <t>2026-09-10T23:44:26.788Z</t>
   </si>
   <si>
     <t>http://adobe.puntos.net.s3-website-us-east-1.amazonaws.com/adobe-partner/personalizacion</t>
+  </si>
+  <si>
+    <t>blog/mi-primer-post.report.json</t>
+  </si>
+  <si>
+    <t>blog/mi-primer-post</t>
+  </si>
+  <si>
+    <t>blog-detail</t>
+  </si>
+  <si>
+    <t>2026-08-25T23:56:20.828Z</t>
+  </si>
+  <si>
+    <t>Titulo 1</t>
+  </si>
+  <si>
+    <t>http://adobe.puntos.net.s3-website-us-east-1.amazonaws.com/blog/mi-primer-post</t>
+  </si>
+  <si>
+    <t>nosotros/quienes-somos.report.json</t>
+  </si>
+  <si>
+    <t>["hero-title","columns-media","columns-media","columns-media","columns-media"]</t>
+  </si>
+  <si>
+    <t>nosotros/quienes-somos</t>
+  </si>
+  <si>
+    <t>institutional</t>
+  </si>
+  <si>
+    <t>2026-08-25T23:56:28.242Z</t>
+  </si>
+  <si>
+    <t>http://adobe.puntos.net.s3-website-us-east-1.amazonaws.com/nosotros/quienes-somos</t>
+  </si>
+  <si>
+    <t>nosotros/storytelling.report.json</t>
+  </si>
+  <si>
+    <t>nosotros/storytelling</t>
+  </si>
+  <si>
+    <t>2026-08-25T23:56:34.594Z</t>
+  </si>
+  <si>
+    <t>http://adobe.puntos.net.s3-website-us-east-1.amazonaws.com/nosotros/storytelling</t>
   </si>
 </sst>
 </file>
@@ -531,7 +612,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="50" customWidth="1"/>
@@ -608,33 +689,33 @@
         <v>11</v>
       </c>
       <c r="E3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" t="s">
         <v>19</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" t="s">
         <v>20</v>
-      </c>
-      <c r="G3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
         <v>22</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>23</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
         <v>24</v>
-      </c>
-      <c r="D4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" t="s">
-        <v>19</v>
       </c>
       <c r="F4" t="s">
         <v>25</v>
@@ -660,94 +741,224 @@
         <v>11</v>
       </c>
       <c r="E5" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="F5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G5" t="s">
         <v>14</v>
       </c>
       <c r="H5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s">
         <v>11</v>
       </c>
       <c r="E6" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="F6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G6" t="s">
         <v>14</v>
       </c>
       <c r="H6" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>
       </c>
       <c r="E7" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="F7" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="G7" t="s">
         <v>14</v>
       </c>
       <c r="H7" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="C8" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D8" t="s">
         <v>11</v>
       </c>
       <c r="E8" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="F8" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="G8" t="s">
         <v>14</v>
       </c>
       <c r="H8" t="s">
-        <v>43</v>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" t="s">
+        <v>48</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" t="s">
+        <v>49</v>
+      </c>
+      <c r="G9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" t="s">
+        <v>52</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F10" t="s">
+        <v>53</v>
+      </c>
+      <c r="G10" t="s">
+        <v>14</v>
+      </c>
+      <c r="H10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>55</v>
+      </c>
+      <c r="B11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" t="s">
+        <v>56</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>57</v>
+      </c>
+      <c r="F11" t="s">
+        <v>58</v>
+      </c>
+      <c r="G11" t="s">
+        <v>59</v>
+      </c>
+      <c r="H11" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C12" t="s">
+        <v>63</v>
+      </c>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>64</v>
+      </c>
+      <c r="F12" t="s">
+        <v>65</v>
+      </c>
+      <c r="G12" t="s">
+        <v>14</v>
+      </c>
+      <c r="H12" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>67</v>
+      </c>
+      <c r="B13" t="s">
+        <v>34</v>
+      </c>
+      <c r="C13" t="s">
+        <v>68</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>64</v>
+      </c>
+      <c r="F13" t="s">
+        <v>69</v>
+      </c>
+      <c r="G13" t="s">
+        <v>14</v>
+      </c>
+      <c r="H13" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>